<commit_message>
[IMP] assets_management: dismissione bene totalmente ammortizzato da più anni
</commit_message>
<xml_diff>
--- a/assets_management/tests/data/account_account.xlsx
+++ b/assets_management/tests/data/account_account.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="98">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -94,7 +94,7 @@
     <t xml:space="preserve">Tax Paid</t>
   </si>
   <si>
-    <t xml:space="preserve">z0bug.bank</t>
+    <t xml:space="preserve">z0bug.coa_bank</t>
   </si>
   <si>
     <t xml:space="preserve">Bank</t>
@@ -103,7 +103,7 @@
     <t xml:space="preserve">account.data_account_type_liquidity</t>
   </si>
   <si>
-    <t xml:space="preserve">z0bug.cash</t>
+    <t xml:space="preserve">z0bug.coa_cash</t>
   </si>
   <si>
     <t xml:space="preserve">Cash</t>
@@ -299,6 +299,12 @@
   </si>
   <si>
     <t xml:space="preserve">Dividends</t>
+  </si>
+  <si>
+    <t xml:space="preserve">z0bug.coa_gc_rc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G/C RC</t>
   </si>
   <si>
     <t xml:space="preserve">z0bug.lp</t>
@@ -541,7 +547,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="53.04"/>
@@ -1190,26 +1196,44 @@
         <v>93</v>
       </c>
       <c r="B38" s="2" t="n">
+        <v>490050</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F38" s="4"/>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B39" s="2" t="n">
         <v>999999</v>
       </c>
-      <c r="C38" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F38" s="4"/>
+      <c r="C39" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Pagina &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Normale"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normale"&amp;12Pagina &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>